<commit_message>
search not verify yet
</commit_message>
<xml_diff>
--- a/resources/testdata/EmployeeData.xlsx
+++ b/resources/testdata/EmployeeData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\racha\eclipse-workspace\Seleniumi-Interview\Selenium_Interview\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DBA24B6-C0DE-41D0-9BC7-EDB6D569FA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51887FBA-8399-4558-9E78-73231A33458C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,12 +41,6 @@
     <t>LastName</t>
   </si>
   <si>
-    <t>Bala</t>
-  </si>
-  <si>
-    <t>Kumar</t>
-  </si>
-  <si>
     <t>Rahul</t>
   </si>
   <si>
@@ -63,6 +57,12 @@
   </si>
   <si>
     <t>Patil</t>
+  </si>
+  <si>
+    <t>bala</t>
+  </si>
+  <si>
+    <t>kumar</t>
   </si>
 </sst>
 </file>
@@ -619,34 +619,34 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>